<commit_message>
chore: atualiza histórico de ordens 2026-07-30
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +469,90 @@
       </c>
       <c r="E2" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="E4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-07-31
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46233</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46233</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46233</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46233</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -553,6 +553,27 @@
       </c>
       <c r="E6" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-03
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,7 +556,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -574,6 +574,69 @@
       </c>
       <c r="E7" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="E8" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>26.75</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>18.85</v>
+      </c>
+      <c r="E10" t="n">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-04
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,7 +577,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -637,6 +637,27 @@
       </c>
       <c r="E10" t="n">
         <v>63</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>27.57</v>
+      </c>
+      <c r="E11" t="n">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-05
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,7 +640,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>46238</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -658,6 +658,27 @@
       </c>
       <c r="E11" t="n">
         <v>28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-06
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,7 +682,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>46239</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,6 +699,48 @@
         <v>53.48</v>
       </c>
       <c r="E13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.789999961853027</v>
+      </c>
+      <c r="E14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>53.47999954223633</v>
+      </c>
+      <c r="E15" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-07
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,7 +829,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -909,6 +909,90 @@
         <v>41.97</v>
       </c>
       <c r="E23" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>27</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="E26" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>41.97</v>
+      </c>
+      <c r="E27" t="n">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-10
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -997,7 +997,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -1141,6 +1141,48 @@
       </c>
       <c r="E34" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>25.32</v>
+      </c>
+      <c r="E35" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="E36" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-11
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1144,7 +1144,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>46244</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>46244</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -1183,6 +1183,27 @@
       </c>
       <c r="E36" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>50.13</v>
+      </c>
+      <c r="E37" t="n">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-14
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,7 +1186,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -1204,6 +1204,48 @@
       </c>
       <c r="E37" t="n">
         <v>45</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="E38" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>17.53</v>
+      </c>
+      <c r="E39" t="n">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-17
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1207,7 +1207,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -1246,6 +1246,48 @@
       </c>
       <c r="E39" t="n">
         <v>63</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="E40" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="E41" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-18
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1249,7 +1249,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -1288,6 +1288,27 @@
       </c>
       <c r="E41" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="E42" t="n">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-19
</commit_message>
<xml_diff>
--- a/historico_ordens.xlsx
+++ b/historico_ordens.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,7 +1291,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -1309,6 +1309,69 @@
       </c>
       <c r="E42" t="n">
         <v>27</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E43" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="E44" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>43.07</v>
+      </c>
+      <c r="E45" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>